<commit_message>
fix(delivery): regenerate acceptance artifacts from honest snapshot
- 新snapshot snap-aaba8a1e3f（顧客2,268・案件2,459・sourceRecordUpdatedAt
  2026-06-29一致を検証。旧snap-df4dca5099はHISTORICAL/SUPERSEDED FOR DELIVERY。
  row-level完全一致は検証不能と明記）から3成果物を単一Snapshotで再生成。
- 出所欄の「更新<取得時刻>」表記をdelivery生成処理のSpec後処理で「取得」へ正規化し、
  freshnessをdataUpdated基準VERY_STALE表記へ（srcコードは無変更）。
- SNAPSHOT_EVIDENCEへSourceごとの行数・列数・列構成SHA-256・
  canonical content SHA-256を追加（生セル値・顧客名不含）。
- 独立検査スクリプトverify-delivery-artifacts.mjs追加（PASS14/FAIL0/UNVERIFIED3を記録）。
- MANIFEST・受入チェックリストを新snapshotへ更新（社長確認欄は全行空欄維持）。

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/受入チェックリスト.xlsx
+++ b/受入チェックリスト.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="119" uniqueCount="107">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="147" uniqueCount="121">
   <si>
     <t>No</t>
   </si>
@@ -43,7 +43,7 @@
     <t>ブラウザでLCC COMMANDが表示される</t>
   </si>
   <si>
-    <t>✅ 開発側クリーン展開でPASS（是正⑤: 起動×2回・health200・err.log 0B）</t>
+    <t>PASS（開発側クリーン展開で1回目・2回目ともPASS。health HTTP 200・server.err.log 0B・bat正常終了）</t>
   </si>
   <si>
     <t>社長確認欄は空欄のまま（社長操作での確認待ち）</t>
@@ -115,7 +115,7 @@
     <t>✅ 再生成・混入ゼロ検査済み</t>
   </si>
   <si>
-    <t>是正⑥: snap-a8bd8e3e57 から再生成・禁止表現機械検査PASS</t>
+    <t>夜間最終走行: snap-aaba8a1e3f から再生成・独立スクリプトで禁止/必須文言検査PASS</t>
   </si>
   <si>
     <t>XLSX生成</t>
@@ -127,7 +127,7 @@
     <t>19列×実案件2,459行+メタデータシート</t>
   </si>
   <si>
-    <t>是正⑥: snap-a8bd8e3e57 から再生成・2,459行・Freshness分離確認</t>
+    <t>夜間最終走行: snap-aaba8a1e3f から再生成・2,459行・非表示シート/外部リンク/名前定義なし</t>
   </si>
   <si>
     <t>PDF生成</t>
@@ -142,7 +142,7 @@
     <t>✅ 再生成済み</t>
   </si>
   <si>
-    <t>是正⑥: snap-a8bd8e3e57 から再生成</t>
+    <t>夜間最終走行: snap-aaba8a1e3f から再生成・3ページ構造正常</t>
   </si>
   <si>
     <t>単一Snapshot</t>
@@ -151,13 +151,13 @@
     <t>3成果物のSnapshot IDを見比べる</t>
   </si>
   <si>
-    <t>同一ID（例: snap-a8bd8e3e57）</t>
+    <t>同一ID（例: snap-aaba8a1e3f）</t>
   </si>
   <si>
     <t>✅ 3点一致を確認</t>
   </si>
   <si>
-    <t>是正⑥再生成分で3点一致を確認</t>
+    <t>3点とも同一Snapshot Objectから生成（成果物ごとの再取得なし）</t>
   </si>
   <si>
     <t>架空顧客</t>
@@ -223,7 +223,7 @@
     <t>サーバー停止</t>
   </si>
   <si>
-    <t>✅ 開発側2回PASS（保存PIDのみ停止・port8787閉塞確認・pid削除）</t>
+    <t>PASS（開発側1回目・2回目ともPASS。保存PIDのみ停止・port8787閉塞・pid削除・他nodeプロセス無影響）</t>
   </si>
   <si>
     <t>社長確認欄は空欄のまま</t>
@@ -271,7 +271,7 @@
     <t>受注残総額: 算出不能（金額確認済0/91件・カバレッジ0%）。0円非表示・value=null・confidence=UNKNOWN</t>
   </si>
   <si>
-    <t>✅ 是正⑥再生成成果物の機械検査で「算出不能」表記を確認（0円表記なし）</t>
+    <t>PASS（再生成成果物の機械検査で「算出不能」表記・0円表記なしを確認）</t>
   </si>
   <si>
     <t>意味検証: Source更新時刻</t>
@@ -298,16 +298,58 @@
     <t/>
   </si>
   <si>
+    <t>開発側: health</t>
+  </si>
+  <si>
+    <t>curl http://localhost:8787/health</t>
+  </si>
+  <si>
+    <t>HTTP 200</t>
+  </si>
+  <si>
+    <t>PASS（クリーン展開スモークで確認）</t>
+  </si>
+  <si>
+    <t>開発側: VUI認証</t>
+  </si>
+  <si>
+    <t>/vui?token=&lt;有効トークン&gt; と無効トークン</t>
+  </si>
+  <si>
+    <t>有効200・無効/なし401</t>
+  </si>
+  <si>
+    <t>PASS</t>
+  </si>
+  <si>
+    <t>開発側: KPI API認証</t>
+  </si>
+  <si>
+    <t>/command/kpi?scope=lcc をAuthorizationヘッダで</t>
+  </si>
+  <si>
+    <t>有効200・無効401</t>
+  </si>
+  <si>
+    <t>開発側: production/Demo隔離</t>
+  </si>
+  <si>
+    <t>/command/health のmodeと/devエンドポイント</t>
+  </si>
+  <si>
+    <t>mode=production・devは無効・Demo fallbackなし</t>
+  </si>
+  <si>
     <t>意味検証: PROVISIONAL候補</t>
   </si>
   <si>
     <t>PPTX/KPIの営業対応表示を見る</t>
   </si>
   <si>
-    <t>「次工程未設定候補 91件（status=contractの意味確認待ち）」表示・確定した営業要対応と表現しない（MEDIUM/WATCH扱い）</t>
-  </si>
-  <si>
-    <t>✅ 是正⑥再生成PPTXのスライド文言で機械確認</t>
+    <t>「次工程未設定候補 91件（status=contractの意味確認待ち）」・MEDIUM・WATCH。確定営業要対応/HIGH表記なし</t>
+  </si>
+  <si>
+    <t>PASS（再生成PPTX全スライドテキストで機械確認）</t>
   </si>
   <si>
     <t>意味検証: Freshness分離</t>
@@ -316,10 +358,10 @@
     <t>成果物のSnapshot欄を見る</t>
   </si>
   <si>
-    <t>sourceRecordUpdatedAt=2026-06-29T09:30:07Z（データ実更新）と snapshotFetchedAt=2026-08-09T15:01:48Z（取得時刻）が別項目で表示される（データ鮮度はVERY_STALE相当=41日超）</t>
-  </si>
-  <si>
-    <t>✅ XLSXメタデータ・PPTX出所スライドで機械確認</t>
+    <t>dataUpdated=2026-06-29T09:30:07Z（Source実更新）とsyncedAt=2026-08-09T15:46:35.585Z（取得時刻）が別項目・VERY_STALE明示・出所欄は「取得」表記（取得時刻を更新と表示しない）</t>
+  </si>
+  <si>
+    <t>PASS（PPTX/XLSXの実テキストで機械確認）</t>
   </si>
   <si>
     <t>総合判定</t>
@@ -718,7 +760,7 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:G26"/>
+  <dimension ref="A1:G30"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
@@ -1190,9 +1232,9 @@
         <v>94</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A26">
-        <v>23</v>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>94</v>
       </c>
       <c r="B26" t="s">
         <v>103</v>
@@ -1204,7 +1246,99 @@
         <v>105</v>
       </c>
       <c r="E26" t="s">
+        <v>102</v>
+      </c>
+      <c r="F26" t="s">
+        <v>94</v>
+      </c>
+      <c r="G26" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>94</v>
+      </c>
+      <c r="B27" t="s">
         <v>106</v>
+      </c>
+      <c r="C27" t="s">
+        <v>107</v>
+      </c>
+      <c r="D27" t="s">
+        <v>108</v>
+      </c>
+      <c r="E27" t="s">
+        <v>102</v>
+      </c>
+      <c r="F27" t="s">
+        <v>94</v>
+      </c>
+      <c r="G27" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>94</v>
+      </c>
+      <c r="B28" t="s">
+        <v>109</v>
+      </c>
+      <c r="C28" t="s">
+        <v>110</v>
+      </c>
+      <c r="D28" t="s">
+        <v>111</v>
+      </c>
+      <c r="E28" t="s">
+        <v>112</v>
+      </c>
+      <c r="F28" t="s">
+        <v>94</v>
+      </c>
+      <c r="G28" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>94</v>
+      </c>
+      <c r="B29" t="s">
+        <v>113</v>
+      </c>
+      <c r="C29" t="s">
+        <v>114</v>
+      </c>
+      <c r="D29" t="s">
+        <v>115</v>
+      </c>
+      <c r="E29" t="s">
+        <v>116</v>
+      </c>
+      <c r="F29" t="s">
+        <v>94</v>
+      </c>
+      <c r="G29" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A30">
+        <v>23</v>
+      </c>
+      <c r="B30" t="s">
+        <v>117</v>
+      </c>
+      <c r="C30" t="s">
+        <v>118</v>
+      </c>
+      <c r="D30" t="s">
+        <v>119</v>
+      </c>
+      <c r="E30" t="s">
+        <v>120</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
docs(delivery): record correction-7 LLM/Memory acceptance (FULLY CONNECTED)
- MANIFEST: applicationCodeCommit=3740ae3・是正⑦履歴・LLM/MEMORY ACCEPTANCE節追加
  （snapshot snap-aaba8a1e3f・成果物3点SHA-256は無変更維持）
- 受入チェックリスト: 是正⑦の開発側確認6行追加（社長確認欄は空欄維持）
- update-checklist-llm.mjs（delivery資材）

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/受入チェックリスト.xlsx
+++ b/受入チェックリスト.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="147" uniqueCount="121">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="189" uniqueCount="144">
   <si>
     <t>No</t>
   </si>
@@ -362,6 +362,75 @@
   </si>
   <si>
     <t>PASS（PPTX/XLSXの実テキストで機械確認）</t>
+  </si>
+  <si>
+    <t>是正⑦: Provider状態</t>
+  </si>
+  <si>
+    <t>/command/providers を見る</t>
+  </si>
+  <si>
+    <t>Anthropic=ACTIVE（実API疎通200）・キー存在だけでACTIVE表示しない・キー情報の露出なし</t>
+  </si>
+  <si>
+    <t>PASS（2026-08-10実機。無効キー時はAUTH_FAILED表示も確認）</t>
+  </si>
+  <si>
+    <t>是正⑦: 一般相談AI</t>
+  </si>
+  <si>
+    <t>「一般論として、部門長会議を30分以内に…」を送る</t>
+  </si>
+  <si>
+    <t>実Anthropic回答・general_reasoning・質問文エコーバックなし・社内事実の捏造なし</t>
+  </si>
+  <si>
+    <t>PASS（2026-08-10実機）</t>
+  </si>
+  <si>
+    <t>是正⑦: production正直Fallback</t>
+  </si>
+  <si>
+    <t>Provider障害時の応答を見る（開発側は無効キー注入で確認済み）</t>
+  </si>
+  <si>
+    <t>「現在、相談AIへ接続できません。Memory検索と社内データ検索は利用できますが…」。mock回答・エコーバック・架空回答なし</t>
+  </si>
+  <si>
+    <t>PASS（合成無効キーでAUTH_FAILED+正直応答を実機確認）</t>
+  </si>
+  <si>
+    <t>是正⑦: Memory想起</t>
+  </si>
+  <si>
+    <t>「私が希望している回答の順番を教えて」を送る</t>
+  </si>
+  <si>
+    <t>memory_search使用・保存済み内容（結論→根拠→次の一手）とEvidence表示</t>
+  </si>
+  <si>
+    <t>PASS（再起動後も同一Memory ID mem-2026-08-09-0）</t>
+  </si>
+  <si>
+    <t>是正⑦: Memory保存先</t>
+  </si>
+  <si>
+    <t>data保存先を確認</t>
+  </si>
+  <si>
+    <t>%LOCALAPPDATA%\LCC_COMMAND\data\lcc-command-local.json（OneDrive外）。旧ファイルはSHA-256一致コピー後も保持</t>
+  </si>
+  <si>
+    <t>是正⑦: 自動Curation</t>
+  </si>
+  <si>
+    <t>「私は、曖昧に賛成されるより…」を覚えてと言わずに送る</t>
+  </si>
+  <si>
+    <t>PREFERENCE候補が自動生成（UNVERIFIED・AUTO・秘密情報なし）</t>
+  </si>
+  <si>
+    <t>PASS（実LLMで mem-2026-08-10-0 生成）</t>
   </si>
   <si>
     <t>総合判定</t>
@@ -760,7 +829,7 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:G30"/>
+  <dimension ref="A1:G36"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
@@ -1324,9 +1393,9 @@
         <v>94</v>
       </c>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A30">
-        <v>23</v>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>94</v>
       </c>
       <c r="B30" t="s">
         <v>117</v>
@@ -1339,6 +1408,144 @@
       </c>
       <c r="E30" t="s">
         <v>120</v>
+      </c>
+      <c r="F30" t="s">
+        <v>94</v>
+      </c>
+      <c r="G30" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>94</v>
+      </c>
+      <c r="B31" t="s">
+        <v>121</v>
+      </c>
+      <c r="C31" t="s">
+        <v>122</v>
+      </c>
+      <c r="D31" t="s">
+        <v>123</v>
+      </c>
+      <c r="E31" t="s">
+        <v>124</v>
+      </c>
+      <c r="F31" t="s">
+        <v>94</v>
+      </c>
+      <c r="G31" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>94</v>
+      </c>
+      <c r="B32" t="s">
+        <v>125</v>
+      </c>
+      <c r="C32" t="s">
+        <v>126</v>
+      </c>
+      <c r="D32" t="s">
+        <v>127</v>
+      </c>
+      <c r="E32" t="s">
+        <v>128</v>
+      </c>
+      <c r="F32" t="s">
+        <v>94</v>
+      </c>
+      <c r="G32" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>94</v>
+      </c>
+      <c r="B33" t="s">
+        <v>129</v>
+      </c>
+      <c r="C33" t="s">
+        <v>130</v>
+      </c>
+      <c r="D33" t="s">
+        <v>131</v>
+      </c>
+      <c r="E33" t="s">
+        <v>132</v>
+      </c>
+      <c r="F33" t="s">
+        <v>94</v>
+      </c>
+      <c r="G33" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>94</v>
+      </c>
+      <c r="B34" t="s">
+        <v>133</v>
+      </c>
+      <c r="C34" t="s">
+        <v>134</v>
+      </c>
+      <c r="D34" t="s">
+        <v>135</v>
+      </c>
+      <c r="E34" t="s">
+        <v>102</v>
+      </c>
+      <c r="F34" t="s">
+        <v>94</v>
+      </c>
+      <c r="G34" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>94</v>
+      </c>
+      <c r="B35" t="s">
+        <v>136</v>
+      </c>
+      <c r="C35" t="s">
+        <v>137</v>
+      </c>
+      <c r="D35" t="s">
+        <v>138</v>
+      </c>
+      <c r="E35" t="s">
+        <v>139</v>
+      </c>
+      <c r="F35" t="s">
+        <v>94</v>
+      </c>
+      <c r="G35" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A36">
+        <v>23</v>
+      </c>
+      <c r="B36" t="s">
+        <v>140</v>
+      </c>
+      <c r="C36" t="s">
+        <v>141</v>
+      </c>
+      <c r="D36" t="s">
+        <v>142</v>
+      </c>
+      <c r="E36" t="s">
+        <v>143</v>
       </c>
     </row>
   </sheetData>

</xml_diff>